<commit_message>
Bill Payment POM Update
</commit_message>
<xml_diff>
--- a/nexus-report/Test_Execution_Report.xlsx
+++ b/nexus-report/Test_Execution_Report.xlsx
@@ -472,15 +472,125 @@
         <v>Bill Payments</v>
       </c>
       <c r="F2" t="str">
-        <v>Electricty Bill Payment Bill Payment</v>
+        <v>Mobile/Telecom Bill Payment Bill Payment</v>
       </c>
       <c r="G2" t="str">
         <v>PASSED</v>
       </c>
       <c r="H2" t="str">
-        <v>29.66</v>
+        <v>26.43</v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Launch browser
+Step 2: Create context
+Step 3: Create page
+Step 4: Navigate to "/banking/login"
+Step 5: Fill "rahul@netbank.com" getByTestId('userId')
+Step 6: Fill "Bank@123" getByTestId('password')
+Step 7: Click getByTestId('loginBtn')
+Step 8: Click getByRole('link', { name: 'Bill Payments' })
+Step 9: Click getByTestId('category-Mobile')
+Step 10: Select option getByTestId('billerProvider')
+Step 11: Fill "870000463" getByTestId('consumerNumber')
+Step 12: Fill "799" getByPlaceholder('Enter amount')
+Step 13: Wait for selector getByTestId('payBillBtn')
+Step 14: Click getByTestId('payBillBtn')
+Step 15: Close context</v>
+      </c>
+      <c r="J2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Embedded in HTML Report</v>
+      </c>
+      <c r="L2" t="str">
+        <v>billPayments.spec.js:16</v>
+      </c>
+      <c r="M2" t="str">
+        <v>10/23/2026, 8:34:52 PM</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TC-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Unspecified</v>
+      </c>
+      <c r="D3" t="str">
+        <v>rahul@netbank.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Bill Payments</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Internet/Broadband Bill Payment Bill Payment</v>
+      </c>
+      <c r="G3" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="H3" t="str">
+        <v>26.46</v>
+      </c>
+      <c r="I3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Launch browser
+Step 2: Create context
+Step 3: Create page
+Step 4: Navigate to "/banking/login"
+Step 5: Fill "rahul@netbank.com" getByTestId('userId')
+Step 6: Fill "Bank@123" getByTestId('password')
+Step 7: Click getByTestId('loginBtn')
+Step 8: Click getByRole('link', { name: 'Bill Payments' })
+Step 9: Click getByTestId('category-Internet')
+Step 10: Select option getByTestId('billerProvider')
+Step 11: Fill "87546463" getByTestId('consumerNumber')
+Step 12: Fill "120" getByPlaceholder('Enter amount')
+Step 13: Wait for selector getByTestId('payBillBtn')
+Step 14: Click getByTestId('payBillBtn')
+Step 15: Close context</v>
+      </c>
+      <c r="J3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Embedded in HTML Report</v>
+      </c>
+      <c r="L3" t="str">
+        <v>billPayments.spec.js:16</v>
+      </c>
+      <c r="M3" t="str">
+        <v>10/23/2026, 8:34:52 PM</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TC-003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Unspecified</v>
+      </c>
+      <c r="D4" t="str">
+        <v>rahul@netbank.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Bill Payments</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Electricty Bill Payment Bill Payment</v>
+      </c>
+      <c r="G4" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="H4" t="str">
+        <v>27.29</v>
+      </c>
+      <c r="I4" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
 Step 2: Create context
 Step 3: Create page
@@ -497,116 +607,6 @@
 Step 14: Click getByTestId('payBillBtn')
 Step 15: Close context</v>
       </c>
-      <c r="J2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Embedded in HTML Report</v>
-      </c>
-      <c r="L2" t="str">
-        <v>BillPayments.spec.js:18</v>
-      </c>
-      <c r="M2" t="str">
-        <v>10/21/2026, 12:35:45 PM</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>TC-002</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Unspecified</v>
-      </c>
-      <c r="D3" t="str">
-        <v>rahul@netbank.com</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Bill Payments</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Mobile/Telecom Bill Payment Bill Payment</v>
-      </c>
-      <c r="G3" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="H3" t="str">
-        <v>28.48</v>
-      </c>
-      <c r="I3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Launch browser
-Step 2: Create context
-Step 3: Create page
-Step 4: Navigate to "/banking/login"
-Step 5: Fill "rahul@netbank.com" getByTestId('userId')
-Step 6: Fill "Bank@123" getByTestId('password')
-Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByRole('link', { name: 'Bill Payments' })
-Step 9: Click getByTestId('category-Mobile')
-Step 10: Select option getByTestId('billerProvider')
-Step 11: Fill "870000463" getByTestId('consumerNumber')
-Step 12: Fill "799" getByPlaceholder('Enter amount')
-Step 13: Wait for selector getByTestId('payBillBtn')
-Step 14: Click getByTestId('payBillBtn')
-Step 15: Close context</v>
-      </c>
-      <c r="J3" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Embedded in HTML Report</v>
-      </c>
-      <c r="L3" t="str">
-        <v>BillPayments.spec.js:18</v>
-      </c>
-      <c r="M3" t="str">
-        <v>10/21/2026, 12:35:45 PM</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>TC-003</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Unspecified</v>
-      </c>
-      <c r="D4" t="str">
-        <v>rahul@netbank.com</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Bill Payments</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Internet/Broadband Bill Payment Bill Payment</v>
-      </c>
-      <c r="G4" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="H4" t="str">
-        <v>30.01</v>
-      </c>
-      <c r="I4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Launch browser
-Step 2: Create context
-Step 3: Create page
-Step 4: Navigate to "/banking/login"
-Step 5: Fill "rahul@netbank.com" getByTestId('userId')
-Step 6: Fill "Bank@123" getByTestId('password')
-Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByRole('link', { name: 'Bill Payments' })
-Step 9: Click getByTestId('category-Internet')
-Step 10: Select option getByTestId('billerProvider')
-Step 11: Fill "87546463" getByTestId('consumerNumber')
-Step 12: Fill "120" getByPlaceholder('Enter amount')
-Step 13: Wait for selector getByTestId('payBillBtn')
-Step 14: Click getByTestId('payBillBtn')
-Step 15: Close context</v>
-      </c>
       <c r="J4" t="str">
         <v>N/A</v>
       </c>
@@ -614,10 +614,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L4" t="str">
-        <v>BillPayments.spec.js:18</v>
+        <v>billPayments.spec.js:16</v>
       </c>
       <c r="M4" t="str">
-        <v>10/21/2026, 12:35:45 PM</v>
+        <v>10/23/2026, 8:34:52 PM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bill Payment POM fix
</commit_message>
<xml_diff>
--- a/nexus-report/Test_Execution_Report.xlsx
+++ b/nexus-report/Test_Execution_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -472,13 +472,13 @@
         <v>Bill Payments</v>
       </c>
       <c r="F2" t="str">
-        <v>Fixed Deposit for 2_Year_Tenure</v>
+        <v>Mobile/Telecom Bill Payment Bill Payment</v>
       </c>
       <c r="G2" t="str">
         <v>PASSED</v>
       </c>
       <c r="H2" t="str">
-        <v>14.10</v>
+        <v>23.33</v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
@@ -488,10 +488,14 @@
 Step 5: Fill "rahul@netbank.com" getByTestId('userId')
 Step 6: Fill "Bank@123" getByTestId('password')
 Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByTestId('nav-fixed-deposits')
-Step 9: Fill "200000" getByTestId('fdAmount')
-Step 10: Click getByTestId('tenure-2yr')
-Step 11: Close context</v>
+Step 8: Click getByRole('link', { name: 'Bill Payments' })
+Step 9: Click getByTestId('category-Mobile')
+Step 10: Select option getByTestId('billerProvider')
+Step 11: Fill "870000463" getByTestId('consumerNumber')
+Step 12: Fill "799" getByPlaceholder('Enter amount')
+Step 13: Wait for selector getByTestId('payBillBtn')
+Step 14: Click getByTestId('payBillBtn')
+Step 15: Close context</v>
       </c>
       <c r="J2" t="str">
         <v>N/A</v>
@@ -500,10 +504,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L2" t="str">
-        <v>fixedDeposit.spec.js:15</v>
+        <v>billPayments.spec.js:15</v>
       </c>
       <c r="M2" t="str">
-        <v>10/24/2026, 12:24:16 PM</v>
+        <v>10/24/2026, 10:58:20 PM</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -523,13 +527,13 @@
         <v>Bill Payments</v>
       </c>
       <c r="F3" t="str">
-        <v>Fixed Deposit for 3_Year_Tenure</v>
+        <v>Electricty Bill Payment Bill Payment</v>
       </c>
       <c r="G3" t="str">
         <v>PASSED</v>
       </c>
       <c r="H3" t="str">
-        <v>14.48</v>
+        <v>23.13</v>
       </c>
       <c r="I3" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
@@ -539,10 +543,14 @@
 Step 5: Fill "rahul@netbank.com" getByTestId('userId')
 Step 6: Fill "Bank@123" getByTestId('password')
 Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByTestId('nav-fixed-deposits')
-Step 9: Fill "200000" getByTestId('fdAmount')
-Step 10: Click getByTestId('tenure-3yr')
-Step 11: Close context</v>
+Step 8: Click getByRole('link', { name: 'Bill Payments' })
+Step 9: Click getByTestId('category-Electricity')
+Step 10: Select option getByTestId('billerProvider')
+Step 11: Fill "87643443" getByTestId('consumerNumber')
+Step 12: Fill "150" getByPlaceholder('Enter amount')
+Step 13: Wait for selector getByTestId('payBillBtn')
+Step 14: Click getByTestId('payBillBtn')
+Step 15: Close context</v>
       </c>
       <c r="J3" t="str">
         <v>N/A</v>
@@ -551,10 +559,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L3" t="str">
-        <v>fixedDeposit.spec.js:15</v>
+        <v>billPayments.spec.js:15</v>
       </c>
       <c r="M3" t="str">
-        <v>10/24/2026, 12:24:18 PM</v>
+        <v>10/24/2026, 10:58:20 PM</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -574,13 +582,13 @@
         <v>Bill Payments</v>
       </c>
       <c r="F4" t="str">
-        <v>Fixed Deposit for 6_Month_Tenure</v>
+        <v>Internet/Broadband Bill Payment Bill Payment</v>
       </c>
       <c r="G4" t="str">
         <v>PASSED</v>
       </c>
       <c r="H4" t="str">
-        <v>16.46</v>
+        <v>23.49</v>
       </c>
       <c r="I4" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
@@ -590,10 +598,14 @@
 Step 5: Fill "rahul@netbank.com" getByTestId('userId')
 Step 6: Fill "Bank@123" getByTestId('password')
 Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByTestId('nav-fixed-deposits')
-Step 9: Fill "200000" getByTestId('fdAmount')
-Step 10: Click getByTestId('tenure-6mo')
-Step 11: Close context</v>
+Step 8: Click getByRole('link', { name: 'Bill Payments' })
+Step 9: Click getByTestId('category-Internet')
+Step 10: Select option getByTestId('billerProvider')
+Step 11: Fill "87546463" getByTestId('consumerNumber')
+Step 12: Fill "120" getByPlaceholder('Enter amount')
+Step 13: Wait for selector getByTestId('payBillBtn')
+Step 14: Click getByTestId('payBillBtn')
+Step 15: Close context</v>
       </c>
       <c r="J4" t="str">
         <v>N/A</v>
@@ -602,116 +614,15 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L4" t="str">
-        <v>fixedDeposit.spec.js:15</v>
+        <v>billPayments.spec.js:15</v>
       </c>
       <c r="M4" t="str">
-        <v>10/24/2026, 12:24:18 PM</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>TC-004</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Unspecified</v>
-      </c>
-      <c r="D5" t="str">
-        <v>rahul@netbank.com</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Bill Payments</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Fixed Deposit for 1_Year_Tenure</v>
-      </c>
-      <c r="G5" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="H5" t="str">
-        <v>15.32</v>
-      </c>
-      <c r="I5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Launch browser
-Step 2: Create context
-Step 3: Create page
-Step 4: Navigate to "/banking/login"
-Step 5: Fill "rahul@netbank.com" getByTestId('userId')
-Step 6: Fill "Bank@123" getByTestId('password')
-Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByTestId('nav-fixed-deposits')
-Step 9: Fill "200000" getByTestId('fdAmount')
-Step 10: Click getByTestId('tenure-1yr')
-Step 11: Close context</v>
-      </c>
-      <c r="J5" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Embedded in HTML Report</v>
-      </c>
-      <c r="L5" t="str">
-        <v>fixedDeposit.spec.js:15</v>
-      </c>
-      <c r="M5" t="str">
-        <v>10/24/2026, 12:24:19 PM</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>TC-005</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Unspecified</v>
-      </c>
-      <c r="D6" t="str">
-        <v>rahul@netbank.com</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Bill Payments</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Fixed Deposit for 5_Year_Tenure</v>
-      </c>
-      <c r="G6" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="H6" t="str">
-        <v>7.41</v>
-      </c>
-      <c r="I6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Create context
-Step 2: Create page
-Step 3: Navigate to "/banking/login"
-Step 4: Fill "rahul@netbank.com" getByTestId('userId')
-Step 5: Fill "Bank@123" getByTestId('password')
-Step 6: Click getByTestId('loginBtn')
-Step 7: Click getByTestId('nav-fixed-deposits')
-Step 8: Fill "200000" getByTestId('fdAmount')
-Step 9: Click getByTestId('tenure-5yr')
-Step 10: Close context</v>
-      </c>
-      <c r="J6" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Embedded in HTML Report</v>
-      </c>
-      <c r="L6" t="str">
-        <v>fixedDeposit.spec.js:15</v>
-      </c>
-      <c r="M6" t="str">
-        <v>10/24/2026, 12:24:23 PM</v>
+        <v>10/24/2026, 10:58:20 PM</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bill Payment fix 1
</commit_message>
<xml_diff>
--- a/nexus-report/Test_Execution_Report.xlsx
+++ b/nexus-report/Test_Execution_Report.xlsx
@@ -472,29 +472,29 @@
         <v>Bill Payments</v>
       </c>
       <c r="F2" t="str">
-        <v>Mobile/Telecom Bill Payment Bill Payment</v>
+        <v>Internet/Broadband Bill Payment Bill Payment</v>
       </c>
       <c r="G2" t="str">
         <v>PASSED</v>
       </c>
       <c r="H2" t="str">
-        <v>23.33</v>
+        <v>17.23</v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
 Step 2: Create context
 Step 3: Create page
-Step 4: Navigate to "/banking/login"
-Step 5: Fill "rahul@netbank.com" getByTestId('userId')
-Step 6: Fill "Bank@123" getByTestId('password')
-Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByRole('link', { name: 'Bill Payments' })
-Step 9: Click getByTestId('category-Mobile')
-Step 10: Select option getByTestId('billerProvider')
-Step 11: Fill "870000463" getByTestId('consumerNumber')
-Step 12: Fill "799" getByPlaceholder('Enter amount')
-Step 13: Wait for selector getByTestId('payBillBtn')
-Step 14: Click getByTestId('payBillBtn')
+Step 4: Navigate — /banking/login
+Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
+Step 6: Fill "Bank@123" — getByTestId('password')
+Step 7: Click — getByTestId('loginBtn')
+Step 8: Click — getByRole('link', { name: 'Bill Payments' })
+Step 9: Click — getByTestId('category-Internet')
+Step 10: Select option — getByTestId('billerProvider')
+Step 11: Fill "87546463" — getByTestId('consumerNumber')
+Step 12: Fill "120" — getByPlaceholder('Enter amount')
+Step 13: Wait for selector — getByTestId('payBillBtn')
+Step 14: Click — getByTestId('payBillBtn')
 Step 15: Close context</v>
       </c>
       <c r="J2" t="str">
@@ -504,10 +504,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L2" t="str">
-        <v>billPayments.spec.js:15</v>
+        <v>payBill.spec.js:15</v>
       </c>
       <c r="M2" t="str">
-        <v>10/24/2026, 10:58:20 PM</v>
+        <v>10/25/2026, 10:01:11 PM</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -533,23 +533,23 @@
         <v>PASSED</v>
       </c>
       <c r="H3" t="str">
-        <v>23.13</v>
+        <v>16.41</v>
       </c>
       <c r="I3" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
 Step 2: Create context
 Step 3: Create page
-Step 4: Navigate to "/banking/login"
-Step 5: Fill "rahul@netbank.com" getByTestId('userId')
-Step 6: Fill "Bank@123" getByTestId('password')
-Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByRole('link', { name: 'Bill Payments' })
-Step 9: Click getByTestId('category-Electricity')
-Step 10: Select option getByTestId('billerProvider')
-Step 11: Fill "87643443" getByTestId('consumerNumber')
-Step 12: Fill "150" getByPlaceholder('Enter amount')
-Step 13: Wait for selector getByTestId('payBillBtn')
-Step 14: Click getByTestId('payBillBtn')
+Step 4: Navigate — /banking/login
+Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
+Step 6: Fill "Bank@123" — getByTestId('password')
+Step 7: Click — getByTestId('loginBtn')
+Step 8: Click — getByRole('link', { name: 'Bill Payments' })
+Step 9: Click — getByTestId('category-Electricity')
+Step 10: Select option — getByTestId('billerProvider')
+Step 11: Fill "87643443" — getByTestId('consumerNumber')
+Step 12: Fill "150" — getByPlaceholder('Enter amount')
+Step 13: Wait for selector — getByTestId('payBillBtn')
+Step 14: Click — getByTestId('payBillBtn')
 Step 15: Close context</v>
       </c>
       <c r="J3" t="str">
@@ -559,10 +559,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L3" t="str">
-        <v>billPayments.spec.js:15</v>
+        <v>payBill.spec.js:15</v>
       </c>
       <c r="M3" t="str">
-        <v>10/24/2026, 10:58:20 PM</v>
+        <v>10/25/2026, 10:01:12 PM</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -582,29 +582,29 @@
         <v>Bill Payments</v>
       </c>
       <c r="F4" t="str">
-        <v>Internet/Broadband Bill Payment Bill Payment</v>
+        <v>Mobile/Telecom Bill Payment Bill Payment</v>
       </c>
       <c r="G4" t="str">
         <v>PASSED</v>
       </c>
       <c r="H4" t="str">
-        <v>23.49</v>
+        <v>17.87</v>
       </c>
       <c r="I4" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
 Step 2: Create context
 Step 3: Create page
-Step 4: Navigate to "/banking/login"
-Step 5: Fill "rahul@netbank.com" getByTestId('userId')
-Step 6: Fill "Bank@123" getByTestId('password')
-Step 7: Click getByTestId('loginBtn')
-Step 8: Click getByRole('link', { name: 'Bill Payments' })
-Step 9: Click getByTestId('category-Internet')
-Step 10: Select option getByTestId('billerProvider')
-Step 11: Fill "87546463" getByTestId('consumerNumber')
-Step 12: Fill "120" getByPlaceholder('Enter amount')
-Step 13: Wait for selector getByTestId('payBillBtn')
-Step 14: Click getByTestId('payBillBtn')
+Step 4: Navigate — /banking/login
+Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
+Step 6: Fill "Bank@123" — getByTestId('password')
+Step 7: Click — getByTestId('loginBtn')
+Step 8: Click — getByRole('link', { name: 'Bill Payments' })
+Step 9: Click — getByTestId('category-Mobile')
+Step 10: Select option — getByTestId('billerProvider')
+Step 11: Fill "870000463" — getByTestId('consumerNumber')
+Step 12: Fill "799" — getByPlaceholder('Enter amount')
+Step 13: Wait for selector — getByTestId('payBillBtn')
+Step 14: Click — getByTestId('payBillBtn')
 Step 15: Close context</v>
       </c>
       <c r="J4" t="str">
@@ -614,10 +614,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L4" t="str">
-        <v>billPayments.spec.js:15</v>
+        <v>payBill.spec.js:15</v>
       </c>
       <c r="M4" t="str">
-        <v>10/24/2026, 10:58:20 PM</v>
+        <v>10/25/2026, 10:01:12 PM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bill Payment Fix 3
</commit_message>
<xml_diff>
--- a/nexus-report/Test_Execution_Report.xlsx
+++ b/nexus-report/Test_Execution_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -472,13 +472,13 @@
         <v>Bill Payments</v>
       </c>
       <c r="F2" t="str">
-        <v>Internet/Broadband Bill Payment Bill Payment</v>
+        <v>Fixed Deposit for 2_Year_Tenure</v>
       </c>
       <c r="G2" t="str">
         <v>PASSED</v>
       </c>
       <c r="H2" t="str">
-        <v>17.23</v>
+        <v>23.70</v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
@@ -488,14 +488,10 @@
 Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
 Step 6: Fill "Bank@123" — getByTestId('password')
 Step 7: Click — getByTestId('loginBtn')
-Step 8: Click — getByRole('link', { name: 'Bill Payments' })
-Step 9: Click — getByTestId('category-Internet')
-Step 10: Select option — getByTestId('billerProvider')
-Step 11: Fill "87546463" — getByTestId('consumerNumber')
-Step 12: Fill "120" — getByPlaceholder('Enter amount')
-Step 13: Wait for selector — getByTestId('payBillBtn')
-Step 14: Click — getByTestId('payBillBtn')
-Step 15: Close context</v>
+Step 8: Click — getByTestId('nav-fixed-deposits')
+Step 9: Fill "200000" — getByTestId('fdAmount')
+Step 10: Click — getByTestId('tenure-2yr')
+Step 11: Close context</v>
       </c>
       <c r="J2" t="str">
         <v>N/A</v>
@@ -504,10 +500,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L2" t="str">
-        <v>payBill.spec.js:15</v>
+        <v>fixedDeposit.spec.js:15</v>
       </c>
       <c r="M2" t="str">
-        <v>10/25/2026, 10:01:11 PM</v>
+        <v>10/25/2026, 10:20:07 PM</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -527,13 +523,13 @@
         <v>Bill Payments</v>
       </c>
       <c r="F3" t="str">
-        <v>Electricty Bill Payment Bill Payment</v>
+        <v>Fixed Deposit for 6_Month_Tenure</v>
       </c>
       <c r="G3" t="str">
         <v>PASSED</v>
       </c>
       <c r="H3" t="str">
-        <v>16.41</v>
+        <v>23.95</v>
       </c>
       <c r="I3" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
@@ -543,14 +539,10 @@
 Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
 Step 6: Fill "Bank@123" — getByTestId('password')
 Step 7: Click — getByTestId('loginBtn')
-Step 8: Click — getByRole('link', { name: 'Bill Payments' })
-Step 9: Click — getByTestId('category-Electricity')
-Step 10: Select option — getByTestId('billerProvider')
-Step 11: Fill "87643443" — getByTestId('consumerNumber')
-Step 12: Fill "150" — getByPlaceholder('Enter amount')
-Step 13: Wait for selector — getByTestId('payBillBtn')
-Step 14: Click — getByTestId('payBillBtn')
-Step 15: Close context</v>
+Step 8: Click — getByTestId('nav-fixed-deposits')
+Step 9: Fill "200000" — getByTestId('fdAmount')
+Step 10: Click — getByTestId('tenure-6mo')
+Step 11: Close context</v>
       </c>
       <c r="J3" t="str">
         <v>N/A</v>
@@ -559,10 +551,10 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L3" t="str">
-        <v>payBill.spec.js:15</v>
+        <v>fixedDeposit.spec.js:15</v>
       </c>
       <c r="M3" t="str">
-        <v>10/25/2026, 10:01:12 PM</v>
+        <v>10/25/2026, 10:20:08 PM</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -582,13 +574,13 @@
         <v>Bill Payments</v>
       </c>
       <c r="F4" t="str">
-        <v>Mobile/Telecom Bill Payment Bill Payment</v>
+        <v>Fixed Deposit for 3_Year_Tenure</v>
       </c>
       <c r="G4" t="str">
         <v>PASSED</v>
       </c>
       <c r="H4" t="str">
-        <v>17.87</v>
+        <v>25.65</v>
       </c>
       <c r="I4" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Launch browser
@@ -598,14 +590,10 @@
 Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
 Step 6: Fill "Bank@123" — getByTestId('password')
 Step 7: Click — getByTestId('loginBtn')
-Step 8: Click — getByRole('link', { name: 'Bill Payments' })
-Step 9: Click — getByTestId('category-Mobile')
-Step 10: Select option — getByTestId('billerProvider')
-Step 11: Fill "870000463" — getByTestId('consumerNumber')
-Step 12: Fill "799" — getByPlaceholder('Enter amount')
-Step 13: Wait for selector — getByTestId('payBillBtn')
-Step 14: Click — getByTestId('payBillBtn')
-Step 15: Close context</v>
+Step 8: Click — getByTestId('nav-fixed-deposits')
+Step 9: Fill "200000" — getByTestId('fdAmount')
+Step 10: Click — getByTestId('tenure-3yr')
+Step 11: Close context</v>
       </c>
       <c r="J4" t="str">
         <v>N/A</v>
@@ -614,15 +602,116 @@
         <v>Embedded in HTML Report</v>
       </c>
       <c r="L4" t="str">
-        <v>payBill.spec.js:15</v>
+        <v>fixedDeposit.spec.js:15</v>
       </c>
       <c r="M4" t="str">
-        <v>10/25/2026, 10:01:12 PM</v>
+        <v>10/25/2026, 10:20:08 PM</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>TC-004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Unspecified</v>
+      </c>
+      <c r="D5" t="str">
+        <v>rahul@netbank.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Bill Payments</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Fixed Deposit for 1_Year_Tenure</v>
+      </c>
+      <c r="G5" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="H5" t="str">
+        <v>24.39</v>
+      </c>
+      <c r="I5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Launch browser
+Step 2: Create context
+Step 3: Create page
+Step 4: Navigate — /banking/login
+Step 5: Fill "rahul@netbank.com" — getByTestId('userId')
+Step 6: Fill "Bank@123" — getByTestId('password')
+Step 7: Click — getByTestId('loginBtn')
+Step 8: Click — getByTestId('nav-fixed-deposits')
+Step 9: Fill "200000" — getByTestId('fdAmount')
+Step 10: Click — getByTestId('tenure-1yr')
+Step 11: Close context</v>
+      </c>
+      <c r="J5" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Embedded in HTML Report</v>
+      </c>
+      <c r="L5" t="str">
+        <v>fixedDeposit.spec.js:15</v>
+      </c>
+      <c r="M5" t="str">
+        <v>10/25/2026, 10:20:08 PM</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>TC-005</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Unspecified</v>
+      </c>
+      <c r="D6" t="str">
+        <v>rahul@netbank.com</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Bill Payments</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Fixed Deposit for 5_Year_Tenure</v>
+      </c>
+      <c r="G6" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="H6" t="str">
+        <v>6.10</v>
+      </c>
+      <c r="I6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Create context
+Step 2: Create page
+Step 3: Navigate — /banking/login
+Step 4: Fill "rahul@netbank.com" — getByTestId('userId')
+Step 5: Fill "Bank@123" — getByTestId('password')
+Step 6: Click — getByTestId('loginBtn')
+Step 7: Click — getByTestId('nav-fixed-deposits')
+Step 8: Fill "200000" — getByTestId('fdAmount')
+Step 9: Click — getByTestId('tenure-5yr')
+Step 10: Close context</v>
+      </c>
+      <c r="J6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Embedded in HTML Report</v>
+      </c>
+      <c r="L6" t="str">
+        <v>fixedDeposit.spec.js:15</v>
+      </c>
+      <c r="M6" t="str">
+        <v>10/25/2026, 10:20:14 PM</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>